<commit_message>
Added new RDF data schemes and visual schemes for environment-table31-35, and fixed XLSX spreadsheet for environment-table31
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table31.xlsx
+++ b/sources/table_normalization/xlsx/environment-table31.xlsx
@@ -500,7 +500,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -557,6 +557,53 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -566,76 +613,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="3" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="16" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -947,7 +952,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1671,14 +1676,14 @@
       <c r="A1" s="1"/>
     </row>
     <row r="2" spans="1:95" ht="31.5" customHeight="1">
-      <c r="A2" s="37" t="s">
+      <c r="A2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="34"/>
-      <c r="L2" s="35"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="35"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
     </row>
     <row r="3" spans="1:95" ht="25.5" customHeight="1">
       <c r="A3" s="5" t="s">
@@ -1693,72 +1698,72 @@
       <c r="H3" s="5"/>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
-      <c r="N3" s="36"/>
-      <c r="O3" s="36"/>
+      <c r="K3" s="53"/>
+      <c r="L3" s="53"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="53"/>
+      <c r="O3" s="53"/>
     </row>
     <row r="4" spans="1:95" ht="40.5" customHeight="1">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="42"/>
-      <c r="J4" s="42"/>
-      <c r="K4" s="45" t="s">
+      <c r="C4" s="56"/>
+      <c r="D4" s="56"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="56"/>
+      <c r="H4" s="56"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="56"/>
+      <c r="K4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="L4" s="46" t="s">
+      <c r="L4" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="M4" s="46"/>
-      <c r="N4" s="54" t="s">
+      <c r="M4" s="58"/>
+      <c r="N4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="O4" s="55"/>
+      <c r="O4" s="59"/>
     </row>
     <row r="5" spans="1:95" ht="41.25" customHeight="1">
-      <c r="A5" s="39"/>
-      <c r="B5" s="43" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="53" t="s">
+      <c r="C5" s="55"/>
+      <c r="D5" s="55"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="55"/>
+      <c r="J5" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="47" t="s">
+      <c r="K5" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="48" t="s">
+      <c r="L5" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="49" t="s">
+      <c r="M5" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="56" t="s">
+      <c r="N5" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="O5" s="57" t="s">
+      <c r="O5" s="49" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:95" ht="58.5" customHeight="1">
-      <c r="A6" s="40"/>
+      <c r="A6" s="54"/>
       <c r="B6" s="7" t="s">
         <v>12</v>
       </c>
@@ -1783,18 +1788,18 @@
       <c r="I6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J6" s="50"/>
-      <c r="K6" s="50" t="s">
+      <c r="J6" s="57"/>
+      <c r="K6" s="43" t="s">
         <v>20</v>
       </c>
-      <c r="L6" s="51" t="s">
+      <c r="L6" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="M6" s="52" t="s">
+      <c r="M6" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="N6" s="58"/>
-      <c r="O6" s="59"/>
+      <c r="N6" s="60"/>
+      <c r="O6" s="61"/>
       <c r="P6" s="8"/>
       <c r="Q6" s="8"/>
       <c r="R6" s="9"/>
@@ -2836,62 +2841,62 @@
       <c r="CQ15" s="3"/>
     </row>
     <row r="16" spans="1:95" ht="39.9" customHeight="1">
-      <c r="A16" s="61" t="s">
+      <c r="A16" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="62">
+      <c r="B16" s="63">
         <f>SUM(B8:B14)</f>
         <v>468</v>
       </c>
-      <c r="C16" s="62">
+      <c r="C16" s="63">
         <f t="shared" ref="C16:I16" si="1">SUM(C8:C14)</f>
         <v>253</v>
       </c>
-      <c r="D16" s="62">
+      <c r="D16" s="63">
         <f t="shared" si="1"/>
         <v>332</v>
       </c>
-      <c r="E16" s="62">
+      <c r="E16" s="63">
         <f t="shared" si="1"/>
         <v>373</v>
       </c>
-      <c r="F16" s="62">
+      <c r="F16" s="63">
         <f t="shared" si="1"/>
         <v>211</v>
       </c>
-      <c r="G16" s="62">
+      <c r="G16" s="63">
         <f t="shared" si="1"/>
         <v>128</v>
       </c>
-      <c r="H16" s="62">
+      <c r="H16" s="63">
         <f t="shared" si="1"/>
         <v>109</v>
       </c>
-      <c r="I16" s="62">
+      <c r="I16" s="63">
         <f t="shared" si="1"/>
         <v>655</v>
       </c>
-      <c r="J16" s="63">
+      <c r="J16" s="64">
         <f>SUM(J8:J14)</f>
         <v>2529</v>
       </c>
-      <c r="K16" s="63">
+      <c r="K16" s="64">
         <f>SUM(K8:K14)</f>
         <v>14</v>
       </c>
-      <c r="L16" s="63">
+      <c r="L16" s="64">
         <f>SUM(L8:L14)</f>
         <v>622</v>
       </c>
-      <c r="M16" s="63">
+      <c r="M16" s="64">
         <f>SUM(M8:M14)</f>
         <v>3165</v>
       </c>
-      <c r="N16" s="63">
+      <c r="N16" s="64">
         <f>SUM(N8:N14)</f>
         <v>3792857</v>
       </c>
-      <c r="O16" s="64">
+      <c r="O16" s="65">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3073,7 +3078,7 @@
       <c r="CP17" s="3"/>
     </row>
     <row r="18" spans="1:94" ht="15.9" customHeight="1">
-      <c r="A18" s="60" t="s">
+      <c r="A18" s="50" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="32"/>
@@ -3267,7 +3272,7 @@
       <c r="CP19" s="3"/>
     </row>
     <row r="20" spans="1:94" ht="15.9" customHeight="1">
-      <c r="A20" s="60" t="s">
+      <c r="A20" s="50" t="s">
         <v>31</v>
       </c>
       <c r="B20" s="32"/>
@@ -3365,7 +3370,7 @@
       <c r="CP20" s="3"/>
     </row>
     <row r="21" spans="1:94" ht="15.9" customHeight="1">
-      <c r="A21" s="60" t="s">
+      <c r="A21" s="50" t="s">
         <v>32</v>
       </c>
       <c r="B21" s="32"/>
@@ -3463,7 +3468,7 @@
       <c r="CP21" s="3"/>
     </row>
     <row r="22" spans="1:94" ht="15.9" customHeight="1">
-      <c r="A22" s="60" t="s">
+      <c r="A22" s="50" t="s">
         <v>33</v>
       </c>
       <c r="B22" s="32"/>

</xml_diff>